<commit_message>
Actualización cronograma y corrección modelo de datos
Cronograma y entregables Proyecto Restaurante (1).xlsx
Actualización cronograma y corrección modelo de datos
</commit_message>
<xml_diff>
--- a/Cronograma y entregables Proyecto Restaurante (1).xlsx
+++ b/Cronograma y entregables Proyecto Restaurante (1).xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2DBA87D-9D83-474B-B273-C51361D814EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{E2DBA87D-9D83-474B-B273-C51361D814EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AFE2C41-C556-43A2-AD5B-B3DD2C35976E}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma General" sheetId="4" r:id="rId1"/>
@@ -1258,23 +1258,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A73E89E-D9A6-11B2-2E7E-B72E07D7A222}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B44A04D3-8F14-0599-D574-FCC9FDE65512}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1290,8 +1290,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="13887450" cy="9991725"/>
+          <a:off x="609600" y="190500"/>
+          <a:ext cx="22459950" cy="12039600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Implementación de la conexión
Implementación de la conexión a la base de datos y actualización de archivos de configuración
</commit_message>
<xml_diff>
--- a/Cronograma y entregables Proyecto Restaurante (1).xlsx
+++ b/Cronograma y entregables Proyecto Restaurante (1).xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30610"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\aplicacioDesa\SIAR\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="8_{E2DBA87D-9D83-474B-B273-C51361D814EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AFE2C41-C556-43A2-AD5B-B3DD2C35976E}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cronograma General" sheetId="4" r:id="rId1"/>
@@ -1001,7 +1006,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1402,7 +1407,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1699,12 +1704,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FBD52BD-D4C3-4D52-97F2-73B82753FB0A}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1731,7 +1736,7 @@
         <v>33.72</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
@@ -1748,7 +1753,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
@@ -1765,7 +1770,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -1782,7 +1787,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
@@ -1799,7 +1804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>16</v>
       </c>
@@ -1816,7 +1821,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>19</v>
       </c>
@@ -1833,7 +1838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>21</v>
       </c>
@@ -1850,7 +1855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>23</v>
       </c>
@@ -1867,7 +1872,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>26</v>
       </c>
@@ -1884,7 +1889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
@@ -1901,7 +1906,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
@@ -1918,7 +1923,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1934,7 +1939,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -1942,7 +1947,7 @@
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>35</v>
       </c>
@@ -1952,7 +1957,7 @@
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -1968,7 +1973,7 @@
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -1984,7 +1989,7 @@
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -2000,7 +2005,7 @@
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>45</v>
       </c>
@@ -2016,7 +2021,7 @@
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -2032,7 +2037,7 @@
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>51</v>
       </c>
@@ -2056,57 +2061,57 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F22EC033-E92B-4BE5-9848-2C1DBDFA24F1}">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="129.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21">
+    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="91.5">
+    <row r="2" spans="1:1" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="21">
+    <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="121.5">
+    <row r="4" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="21">
+    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A5" s="12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30.75">
+    <row r="6" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="21">
+    <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="106.5">
+    <row r="8" spans="1:1" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="21">
+    <row r="9" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="290.25">
+    <row r="10" spans="1:1" ht="285" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>62</v>
       </c>
@@ -2119,13 +2124,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="108" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>63</v>
       </c>
@@ -2136,7 +2141,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>66</v>
       </c>
@@ -2147,7 +2152,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>69</v>
       </c>
@@ -2158,7 +2163,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>71</v>
       </c>
@@ -2169,7 +2174,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>73</v>
       </c>
@@ -2180,7 +2185,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>76</v>
       </c>
@@ -2191,7 +2196,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>78</v>
       </c>
@@ -2202,7 +2207,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>81</v>
       </c>
@@ -2213,7 +2218,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>83</v>
       </c>
@@ -2224,7 +2229,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>85</v>
       </c>
@@ -2235,7 +2240,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>88</v>
       </c>
@@ -2254,14 +2259,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A30E17-F6D9-40BF-ADF5-99B056D60119}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>63</v>
       </c>
@@ -2272,7 +2277,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>93</v>
       </c>
@@ -2283,7 +2288,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>96</v>
       </c>
@@ -2294,7 +2299,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>98</v>
       </c>
@@ -2305,7 +2310,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>101</v>
       </c>
@@ -2316,7 +2321,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>103</v>
       </c>
@@ -2327,7 +2332,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>105</v>
       </c>
@@ -2338,7 +2343,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>108</v>
       </c>
@@ -2349,7 +2354,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>110</v>
       </c>
@@ -2360,7 +2365,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>112</v>
       </c>
@@ -2371,7 +2376,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>114</v>
       </c>
@@ -2382,7 +2387,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>116</v>
       </c>
@@ -2393,7 +2398,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>118</v>
       </c>
@@ -2404,7 +2409,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>121</v>
       </c>
@@ -2424,13 +2429,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D83E73D-3A8A-4AC0-9C80-3B3E1179B605}">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="67.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="92.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>63</v>
       </c>
@@ -2444,7 +2449,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>125</v>
       </c>
@@ -2458,7 +2463,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>129</v>
       </c>
@@ -2472,7 +2477,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>133</v>
       </c>
@@ -2486,7 +2491,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>137</v>
       </c>
@@ -2500,7 +2505,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>141</v>
       </c>
@@ -2514,7 +2519,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>145</v>
       </c>
@@ -2528,7 +2533,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>149</v>
       </c>
@@ -2542,7 +2547,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>153</v>
       </c>
@@ -2550,7 +2555,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>155</v>
       </c>
@@ -2558,7 +2563,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>157</v>
       </c>
@@ -2566,7 +2571,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>159</v>
       </c>
@@ -2582,7 +2587,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D62219-973C-4B76-973C-EBB00D2A019E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2592,7 +2597,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71CA6DD7-1E1D-4E98-9C07-0E9FDF3D8A7F}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2602,7 +2607,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7065940-5F3C-4514-AE4F-FAB8AD2805BA}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2612,7 +2617,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D98718C2-2990-446F-9FC6-6901F350EE06}">
   <dimension ref="A1:F72"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2622,7 +2627,7 @@
     <col min="6" max="6" width="78.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>161</v>
       </c>
@@ -2642,7 +2647,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>167</v>
       </c>
@@ -2662,7 +2667,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
         <v>167</v>
       </c>
@@ -2682,7 +2687,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
         <v>167</v>
       </c>
@@ -2702,7 +2707,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
         <v>181</v>
       </c>
@@ -2722,7 +2727,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>181</v>
       </c>
@@ -2742,7 +2747,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
         <v>181</v>
       </c>
@@ -2762,7 +2767,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>181</v>
       </c>
@@ -2782,7 +2787,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
         <v>181</v>
       </c>
@@ -2802,7 +2807,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>181</v>
       </c>
@@ -2822,7 +2827,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>181</v>
       </c>
@@ -2842,7 +2847,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
         <v>198</v>
       </c>
@@ -2862,7 +2867,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>198</v>
       </c>
@@ -2882,7 +2887,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>198</v>
       </c>
@@ -2902,7 +2907,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>198</v>
       </c>
@@ -2922,7 +2927,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>198</v>
       </c>
@@ -2942,7 +2947,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
         <v>198</v>
       </c>
@@ -2962,7 +2967,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
         <v>198</v>
       </c>
@@ -2982,7 +2987,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>213</v>
       </c>
@@ -3002,7 +3007,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>213</v>
       </c>
@@ -3022,7 +3027,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
         <v>213</v>
       </c>
@@ -3042,7 +3047,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
         <v>213</v>
       </c>
@@ -3062,7 +3067,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
         <v>221</v>
       </c>
@@ -3082,7 +3087,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
         <v>221</v>
       </c>
@@ -3102,7 +3107,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
         <v>221</v>
       </c>
@@ -3122,7 +3127,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>221</v>
       </c>
@@ -3142,7 +3147,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>221</v>
       </c>
@@ -3162,7 +3167,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
         <v>221</v>
       </c>
@@ -3182,7 +3187,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
         <v>221</v>
       </c>
@@ -3202,7 +3207,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>235</v>
       </c>
@@ -3222,7 +3227,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>235</v>
       </c>
@@ -3242,7 +3247,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
         <v>235</v>
       </c>
@@ -3262,7 +3267,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>235</v>
       </c>
@@ -3282,7 +3287,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>241</v>
       </c>
@@ -3302,7 +3307,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
         <v>241</v>
       </c>
@@ -3322,7 +3327,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>241</v>
       </c>
@@ -3342,7 +3347,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>241</v>
       </c>
@@ -3362,7 +3367,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>241</v>
       </c>
@@ -3382,7 +3387,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>241</v>
       </c>
@@ -3402,7 +3407,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
         <v>241</v>
       </c>
@@ -3422,7 +3427,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>254</v>
       </c>
@@ -3442,7 +3447,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
         <v>254</v>
       </c>
@@ -3462,7 +3467,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>254</v>
       </c>
@@ -3482,7 +3487,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
         <v>254</v>
       </c>
@@ -3502,7 +3507,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>254</v>
       </c>
@@ -3522,7 +3527,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
         <v>254</v>
       </c>
@@ -3542,7 +3547,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
         <v>254</v>
       </c>
@@ -3562,7 +3567,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
         <v>265</v>
       </c>
@@ -3582,7 +3587,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
         <v>265</v>
       </c>
@@ -3602,7 +3607,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
         <v>265</v>
       </c>
@@ -3622,7 +3627,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
         <v>265</v>
       </c>
@@ -3642,7 +3647,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
         <v>265</v>
       </c>
@@ -3662,7 +3667,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
         <v>265</v>
       </c>
@@ -3682,7 +3687,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>265</v>
       </c>
@@ -3702,7 +3707,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
         <v>279</v>
       </c>
@@ -3722,7 +3727,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
         <v>279</v>
       </c>
@@ -3742,7 +3747,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
         <v>279</v>
       </c>
@@ -3762,7 +3767,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
         <v>279</v>
       </c>
@@ -3782,7 +3787,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
         <v>279</v>
       </c>
@@ -3802,7 +3807,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
         <v>279</v>
       </c>
@@ -3822,7 +3827,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
         <v>279</v>
       </c>
@@ -3842,7 +3847,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
         <v>279</v>
       </c>
@@ -3862,7 +3867,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="16" t="s">
         <v>279</v>
       </c>
@@ -3882,7 +3887,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
         <v>279</v>
       </c>
@@ -3902,7 +3907,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="16" t="s">
         <v>296</v>
       </c>
@@ -3922,7 +3927,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="15" t="s">
         <v>296</v>
       </c>
@@ -3942,7 +3947,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="16" t="s">
         <v>296</v>
       </c>
@@ -3962,7 +3967,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="15" t="s">
         <v>300</v>
       </c>
@@ -3982,7 +3987,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="16" t="s">
         <v>300</v>
       </c>
@@ -4002,7 +4007,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
         <v>300</v>
       </c>
@@ -4022,7 +4027,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="16" t="s">
         <v>300</v>
       </c>
@@ -4042,7 +4047,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
         <v>300</v>
       </c>

</xml_diff>